<commit_message>
Fix COR stats fetching and editable Weekly Progress tab
</commit_message>
<xml_diff>
--- a/backend/src/templates/weekly_report_template.xlsx
+++ b/backend/src/templates/weekly_report_template.xlsx
@@ -7,16 +7,17 @@
     <sheet sheetId="1" name="SUMMARY" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="SOW" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="SCHEDULE" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="TRANSMITTAL LOG" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="RFI LOG" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="CDRFI LOG" state="visible" r:id="rId9"/>
+    <sheet sheetId="4" name="COR" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="TRANSMITTAL LOG" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="RFI LOG" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="CDRFI LOG" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
   <si>
     <t>Weekly Project Progress Report</t>
   </si>
@@ -97,6 +98,18 @@
   </si>
   <si>
     <t>Actual Fab</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Pending</t>
   </si>
   <si>
     <t>Transmittal No</t>
@@ -506,7 +519,7 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -555,6 +568,55 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
@@ -594,7 +656,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2039,6 +2101,211 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="4" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="15"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="15"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -2063,16 +2330,16 @@
         <v>15</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>20</v>
@@ -2336,406 +2603,6 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J30"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="30" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
-    <col min="10" max="10" width="30" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B1"/>
-      <c r="C1"/>
-      <c r="D1"/>
-      <c r="E1"/>
-      <c r="F1"/>
-      <c r="G1"/>
-      <c r="H1"/>
-      <c r="I1"/>
-      <c r="J1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="H2" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="14" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A23" s="15"/>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="15"/>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
-      <c r="J27" s="15"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="15"/>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
-      <c r="J30" s="15"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2767,25 +2634,25 @@
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>36</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>37</v>
       </c>
       <c r="C2" s="14" t="s">
         <v>21</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F2" s="14" t="s">
         <v>20</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H2" s="14" t="s">
         <v>16</v>
@@ -3141,4 +3008,404 @@
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J30"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="30" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="30" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="60" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+      <c r="F1"/>
+      <c r="G1"/>
+      <c r="H1"/>
+      <c r="I1"/>
+      <c r="J1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="F2" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="15"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="15"/>
+      <c r="E21" s="15"/>
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="15"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
+      <c r="I23" s="15"/>
+      <c r="J23" s="15"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="15"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
+      <c r="I25" s="15"/>
+      <c r="J25" s="15"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="15"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+      <c r="I28" s="15"/>
+      <c r="J28" s="15"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="15"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+      <c r="I30" s="15"/>
+      <c r="J30" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>